<commit_message>
Mass Mailing  using nodemailer
</commit_message>
<xml_diff>
--- a/Backend/bookings.xlsx
+++ b/Backend/bookings.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -424,7 +424,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>6/8/2025, 9:27:44 pm</v>
+        <v>9/8/2025, 10:58:03 pm</v>
       </c>
       <c r="B2" t="str">
         <v>K ADARSH REDDY</v>
@@ -436,18 +436,45 @@
         <v>+918143154845</v>
       </c>
       <c r="E2" t="str">
-        <v>2025-08-13</v>
+        <v>2025-08-26</v>
       </c>
       <c r="F2" t="str">
+        <v>morning</v>
+      </c>
+      <c r="G2" t="str">
+        <v>....</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>9/8/2025, 11:18:44 pm</v>
+      </c>
+      <c r="B3" t="str">
+        <v>K ADARSH REDDY</v>
+      </c>
+      <c r="C3" t="str">
+        <v>k.adarsh2106@gmail.com</v>
+      </c>
+      <c r="D3" t="str">
+        <v>+918143154845</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2025-08-26</v>
+      </c>
+      <c r="F3" t="str">
         <v>afternoon</v>
       </c>
-      <c r="G2" t="str">
-        <v>...</v>
+      <c r="G3" t="str">
+        <v>hi..</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>